<commit_message>
Webhook e id spa separados. Relatorio
</commit_message>
<xml_diff>
--- a/HorasEad.xlsx
+++ b/HorasEad.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\_adriano\Projetos\Tarefas no Bitrix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C80995A-42E2-4ADD-BB0B-160529103075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B154312-81D9-4327-957B-54CF1F0A6010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25080" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{535172B3-0454-4411-AC82-A02FDE185FD8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{535172B3-0454-4411-AC82-A02FDE185FD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>CODIGO UC</t>
   </si>
@@ -53,21 +53,6 @@
     <t>2026-02</t>
   </si>
   <si>
-    <t>0023581</t>
-  </si>
-  <si>
-    <t>DIREITO DO TRABALHO II</t>
-  </si>
-  <si>
-    <t>357902. fazer +35h</t>
-  </si>
-  <si>
-    <t>boris@feevale.br</t>
-  </si>
-  <si>
-    <t>Boris Chechi de Assis</t>
-  </si>
-  <si>
     <t>NÍVEL DE ENSINO</t>
   </si>
   <si>
@@ -77,45 +62,12 @@
     <t>SEMIPRESENCIAL</t>
   </si>
   <si>
-    <t>METODOLOGIA PROJETUAL PARA MODA</t>
-  </si>
-  <si>
-    <t>360564 e fazer +30h</t>
-  </si>
-  <si>
-    <t>Joeline Maciel Lopes</t>
-  </si>
-  <si>
-    <t>joeline@feevale.br</t>
-  </si>
-  <si>
-    <t>0060011</t>
-  </si>
-  <si>
-    <t>ABORDAGEM QUIROPRÁTICA DA COLUNA LOMBO PÉLVICA</t>
-  </si>
-  <si>
-    <t>362078 - APROVEITAR E ELABORAR 25H PARA 202602</t>
-  </si>
-  <si>
-    <t>0018136</t>
-  </si>
-  <si>
-    <t>Danilo Messa da Silva</t>
-  </si>
-  <si>
-    <t>danilo@feevale.br</t>
-  </si>
-  <si>
     <t>CH TOTAL</t>
   </si>
   <si>
     <t>CURSO</t>
   </si>
   <si>
-    <t>MODA</t>
-  </si>
-  <si>
     <t>DIREITO</t>
   </si>
   <si>
@@ -138,6 +90,30 @@
   </si>
   <si>
     <t>INSTITUTO</t>
+  </si>
+  <si>
+    <t>00001A</t>
+  </si>
+  <si>
+    <t>TESTE 06</t>
+  </si>
+  <si>
+    <t>TEORICO PRÁTICO EAD</t>
+  </si>
+  <si>
+    <t>0082515</t>
+  </si>
+  <si>
+    <t>Adriano Martins Rodrigues</t>
+  </si>
+  <si>
+    <t>adrianomr@feevale.br</t>
+  </si>
+  <si>
+    <t>000005. fazer +35h</t>
+  </si>
+  <si>
+    <t>ICS</t>
   </si>
 </sst>
 </file>
@@ -623,7 +599,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" style="5" customWidth="1"/>
-    <col min="2" max="2" width="11" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" style="17" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="46.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.28515625" style="17" customWidth="1"/>
@@ -637,169 +613,121 @@
   <sheetData>
     <row r="1" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="15" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="I1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="J1" s="12" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K1" s="12" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="L1" s="12" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="M1" s="12" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="N1" s="12" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3">
-        <v>422960</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="3"/>
+      <c r="B2" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>20</v>
+      </c>
       <c r="E2" s="4">
         <v>45</v>
       </c>
-      <c r="F2" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I2" s="3" t="s">
+      <c r="F2" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" s="6" t="s">
         <v>7</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>12</v>
       </c>
       <c r="L2" s="1">
         <v>80</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="N2" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3">
-        <v>424370</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="3"/>
       <c r="D3" s="3"/>
-      <c r="E3" s="4">
-        <v>45</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="L3" s="1">
-        <v>80</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>25</v>
-      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3">
-        <v>420220</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="3"/>
       <c r="D4" s="3"/>
-      <c r="E4" s="4">
-        <v>45</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="L4" s="1">
-        <v>80</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>25</v>
-      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="6"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
       <c r="E5" s="11"/>
@@ -812,7 +740,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="6"/>
+      <c r="B6" s="16"/>
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
       <c r="E6" s="11"/>
@@ -825,7 +753,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="6"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
       <c r="E7" s="11"/>
@@ -838,7 +766,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="6"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
       <c r="E8" s="11"/>
@@ -851,7 +779,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="6"/>
+      <c r="B9" s="16"/>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
       <c r="E9" s="11"/>
@@ -864,7 +792,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="6"/>
+      <c r="B10" s="16"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
       <c r="E10" s="11"/>
@@ -877,7 +805,7 @@
     </row>
     <row r="11" spans="1:14" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
+      <c r="B11" s="16"/>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
       <c r="E11" s="11"/>
@@ -890,7 +818,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="6"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
       <c r="E12" s="11"/>
@@ -903,7 +831,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="6"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
       <c r="E13" s="11"/>
@@ -916,7 +844,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="6"/>
+      <c r="B14" s="16"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
       <c r="E14" s="11"/>
@@ -929,7 +857,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="3"/>
+      <c r="B15" s="13"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="4"/>
@@ -941,7 +869,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="3"/>
+      <c r="B16" s="13"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="4"/>
@@ -953,7 +881,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="3"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="4"/>
@@ -965,7 +893,7 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="3"/>
+      <c r="B18" s="13"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="4"/>
@@ -977,7 +905,7 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="3"/>
+      <c r="B19" s="13"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="4"/>
@@ -989,7 +917,7 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="3"/>
+      <c r="B20" s="13"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="4"/>
@@ -1001,7 +929,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="3"/>
+      <c r="B21" s="13"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="4"/>
@@ -1013,7 +941,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="3"/>
+      <c r="B22" s="13"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="4"/>
@@ -1025,7 +953,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="3"/>
+      <c r="B23" s="13"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="4"/>
@@ -1037,7 +965,7 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="3"/>
+      <c r="B24" s="13"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="4"/>
@@ -1049,7 +977,7 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="3"/>
+      <c r="B25" s="13"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="4"/>
@@ -1061,7 +989,7 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="3"/>
+      <c r="B26" s="13"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="4"/>
@@ -1073,7 +1001,7 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="3"/>
+      <c r="B27" s="13"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="4"/>
@@ -1085,7 +1013,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="3"/>
+      <c r="B28" s="13"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="4"/>
@@ -1097,7 +1025,7 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
+      <c r="B29" s="13"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="4"/>
@@ -1109,7 +1037,7 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="3"/>
+      <c r="B30" s="13"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="4"/>
@@ -1121,7 +1049,7 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
-      <c r="B31" s="3"/>
+      <c r="B31" s="13"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="4"/>
@@ -1133,7 +1061,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
-      <c r="B32" s="3"/>
+      <c r="B32" s="13"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>
@@ -1145,7 +1073,7 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
-      <c r="B33" s="3"/>
+      <c r="B33" s="13"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="4"/>
@@ -1157,7 +1085,7 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
-      <c r="B34" s="3"/>
+      <c r="B34" s="13"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="4"/>

</xml_diff>